<commit_message>
Show 원/%/시간 units in simulation workbook
Percentages are stored as x100 with a literal % suffix and amounts use a
원 suffix, so values read correctly even in viewers that ignore Excel
number formats.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019fqrWohtTSxpdk7nNCRMqp
</commit_message>
<xml_diff>
--- a/baemin_analysis/샵인샵_수익시뮬레이션.xlsx
+++ b/baemin_analysis/샵인샵_수익시뮬레이션.xlsx
@@ -19,8 +19,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
+  <numFmts count="5">
+    <numFmt numFmtId="164" formatCode="#,##0&quot;원&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0&quot;시간&quot;"/>
+    <numFmt numFmtId="166" formatCode="0.0&quot;%&quot;"/>
+    <numFmt numFmtId="167" formatCode="0&quot;시간&quot;"/>
+    <numFmt numFmtId="168" formatCode="0&quot;건/일&quot;"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -72,17 +76,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -640,19 +647,19 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>알바 근무시간 (h/월)</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
+          <t>알바 근무시간 (월)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
         <v>160</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="5" t="n">
         <v>310</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" s="5" t="n">
         <v>310</v>
       </c>
-      <c r="E10" s="3" t="n">
+      <c r="E10" s="5" t="n">
         <v>430</v>
       </c>
     </row>
@@ -681,16 +688,16 @@
           <t>영업이익 (사장 몫, 세전)</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B12" s="6" t="n">
         <v>248419</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="6" t="n">
         <v>1069628</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="6" t="n">
         <v>3825837</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="6" t="n">
         <v>5952783</v>
       </c>
     </row>
@@ -700,16 +707,16 @@
           <t>사장 인건비 300만원 차감 후</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n">
+      <c r="B13" s="7" t="n">
         <v>-2751581</v>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="7" t="n">
         <v>-1930372</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="6" t="n">
         <v>825837</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="6" t="n">
         <v>2952783</v>
       </c>
     </row>
@@ -719,17 +726,17 @@
           <t>공헌이익률</t>
         </is>
       </c>
-      <c r="B14" s="7" t="n">
-        <v>0.2982177571940922</v>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>0.2982177571940922</v>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>0.2982177571940922</v>
-      </c>
-      <c r="E14" s="7" t="n">
-        <v>0.2982177571940922</v>
+      <c r="B14" s="8" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>29.8</v>
       </c>
     </row>
     <row r="15">
@@ -738,17 +745,17 @@
           <t>영업이익률</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
-        <v>0.01343926498151806</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0.03857738669785088</v>
-      </c>
-      <c r="D15" s="7" t="n">
-        <v>0.1034874793219112</v>
-      </c>
-      <c r="E15" s="7" t="n">
-        <v>0.1207654297304201</v>
+      <c r="B15" s="8" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>12.1</v>
       </c>
     </row>
   </sheetData>
@@ -847,8 +854,8 @@
           <t>김치찜 (3대천왕)</t>
         </is>
       </c>
-      <c r="B2" s="7" t="n">
-        <v>0.35</v>
+      <c r="B2" s="8" t="n">
+        <v>35</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>19967</v>
@@ -862,8 +869,8 @@
       <c r="F2" s="3" t="n">
         <v>5700</v>
       </c>
-      <c r="G2" s="7" t="n">
-        <v>0.2854989282208466</v>
+      <c r="G2" s="8" t="n">
+        <v>28.5</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>2105</v>
@@ -880,8 +887,8 @@
       <c r="L2" s="3" t="n">
         <v>6102</v>
       </c>
-      <c r="M2" s="7" t="n">
-        <v>0.3217365712719066</v>
+      <c r="M2" s="8" t="n">
+        <v>32.2</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -895,8 +902,8 @@
           <t>제육덮밥 (제육대가)</t>
         </is>
       </c>
-      <c r="B3" s="7" t="n">
-        <v>0.3</v>
+      <c r="B3" s="8" t="n">
+        <v>30</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>15000</v>
@@ -910,8 +917,8 @@
       <c r="F3" s="3" t="n">
         <v>4950</v>
       </c>
-      <c r="G3" s="7" t="n">
-        <v>0.33</v>
+      <c r="G3" s="8" t="n">
+        <v>33</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>1554</v>
@@ -928,8 +935,8 @@
       <c r="L3" s="3" t="n">
         <v>3036</v>
       </c>
-      <c r="M3" s="7" t="n">
-        <v>0.2168571428571429</v>
+      <c r="M3" s="8" t="n">
+        <v>21.7</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -943,8 +950,8 @@
           <t>닭발 (30년 불멸의 닭발)</t>
         </is>
       </c>
-      <c r="B4" s="7" t="n">
-        <v>0.2</v>
+      <c r="B4" s="8" t="n">
+        <v>20</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>28000</v>
@@ -958,8 +965,8 @@
       <c r="F4" s="3" t="n">
         <v>9240</v>
       </c>
-      <c r="G4" s="7" t="n">
-        <v>0.33</v>
+      <c r="G4" s="8" t="n">
+        <v>33</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>2886</v>
@@ -976,8 +983,8 @@
       <c r="L4" s="3" t="n">
         <v>8634</v>
       </c>
-      <c r="M4" s="7" t="n">
-        <v>0.3320769230769231</v>
+      <c r="M4" s="8" t="n">
+        <v>33.2</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -991,8 +998,8 @@
           <t>곱도리탕 (진곱도리탕)</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
-        <v>0.15</v>
+      <c r="B5" s="8" t="n">
+        <v>15</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>32000</v>
@@ -1006,8 +1013,8 @@
       <c r="F5" s="3" t="n">
         <v>12160</v>
       </c>
-      <c r="G5" s="7" t="n">
-        <v>0.38</v>
+      <c r="G5" s="8" t="n">
+        <v>38</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>3330</v>
@@ -1024,8 +1031,8 @@
       <c r="L5" s="3" t="n">
         <v>9010</v>
       </c>
-      <c r="M5" s="7" t="n">
-        <v>0.3003333333333333</v>
+      <c r="M5" s="8" t="n">
+        <v>30</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -1118,7 +1125,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>[한그릇] 삼겹듬뿍 김치찜</t>
         </is>
@@ -1141,8 +1148,8 @@
       <c r="G2" s="3" t="n">
         <v>4180</v>
       </c>
-      <c r="H2" s="7" t="n">
-        <v>0.3483333333333333</v>
+      <c r="H2" s="8" t="n">
+        <v>34.8</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>900</v>
@@ -1156,12 +1163,12 @@
       <c r="L2" s="3" t="n">
         <v>1951</v>
       </c>
-      <c r="M2" s="7" t="n">
-        <v>0.1773636363636364</v>
+      <c r="M2" s="8" t="n">
+        <v>17.7</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>[1.5인분] 삼겹듬뿍 김치찜</t>
         </is>
@@ -1184,8 +1191,8 @@
       <c r="G3" s="3" t="n">
         <v>6023</v>
       </c>
-      <c r="H3" s="7" t="n">
-        <v>0.4042281879194631</v>
+      <c r="H3" s="8" t="n">
+        <v>40.4</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>900</v>
@@ -1199,12 +1206,12 @@
       <c r="L3" s="3" t="n">
         <v>3678</v>
       </c>
-      <c r="M3" s="7" t="n">
-        <v>0.2646115107913669</v>
+      <c r="M3" s="8" t="n">
+        <v>26.5</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>삼겹듬뿍 2~3인</t>
         </is>
@@ -1227,8 +1234,8 @@
       <c r="G4" s="3" t="n">
         <v>11999</v>
       </c>
-      <c r="H4" s="7" t="n">
-        <v>0.4460594795539033</v>
+      <c r="H4" s="8" t="n">
+        <v>44.6</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>900</v>
@@ -1242,12 +1249,12 @@
       <c r="L4" s="3" t="n">
         <v>9174</v>
       </c>
-      <c r="M4" s="7" t="n">
-        <v>0.3542123552123552</v>
+      <c r="M4" s="8" t="n">
+        <v>35.4</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>삼겹듬뿍 3~4인</t>
         </is>
@@ -1270,8 +1277,8 @@
       <c r="G5" s="3" t="n">
         <v>15796</v>
       </c>
-      <c r="H5" s="7" t="n">
-        <v>0.4449577464788733</v>
+      <c r="H5" s="8" t="n">
+        <v>44.5</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>900</v>
@@ -1285,12 +1292,12 @@
       <c r="L5" s="3" t="n">
         <v>12628</v>
       </c>
-      <c r="M5" s="7" t="n">
-        <v>0.3660144927536232</v>
+      <c r="M5" s="8" t="n">
+        <v>36.6</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>1.5인분 스팸폭탄</t>
         </is>
@@ -1313,8 +1320,8 @@
       <c r="G6" s="3" t="n">
         <v>6448</v>
       </c>
-      <c r="H6" s="7" t="n">
-        <v>0.432751677852349</v>
+      <c r="H6" s="8" t="n">
+        <v>43.3</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>900</v>
@@ -1328,12 +1335,12 @@
       <c r="L6" s="3" t="n">
         <v>4103</v>
       </c>
-      <c r="M6" s="7" t="n">
-        <v>0.2951870503597123</v>
+      <c r="M6" s="8" t="n">
+        <v>29.5</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>스팸폭탄 2~3인</t>
         </is>
@@ -1356,8 +1363,8 @@
       <c r="G7" s="3" t="n">
         <v>13914</v>
       </c>
-      <c r="H7" s="7" t="n">
-        <v>0.5250566037735849</v>
+      <c r="H7" s="8" t="n">
+        <v>52.5</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>900</v>
@@ -1371,12 +1378,12 @@
       <c r="L7" s="3" t="n">
         <v>11104</v>
       </c>
-      <c r="M7" s="7" t="n">
-        <v>0.4354705882352941</v>
+      <c r="M7" s="8" t="n">
+        <v>43.5</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>스팸폭탄 3~4인</t>
         </is>
@@ -1399,8 +1406,8 @@
       <c r="G8" s="3" t="n">
         <v>17618</v>
       </c>
-      <c r="H8" s="7" t="n">
-        <v>0.525910447761194</v>
+      <c r="H8" s="8" t="n">
+        <v>52.6</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>900</v>
@@ -1414,12 +1421,12 @@
       <c r="L8" s="3" t="n">
         <v>14530</v>
       </c>
-      <c r="M8" s="7" t="n">
-        <v>0.4470615384615385</v>
+      <c r="M8" s="8" t="n">
+        <v>44.7</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>1.5인분 우삼겹</t>
         </is>
@@ -1442,8 +1449,8 @@
       <c r="G9" s="3" t="n">
         <v>5448</v>
       </c>
-      <c r="H9" s="7" t="n">
-        <v>0.3656375838926175</v>
+      <c r="H9" s="8" t="n">
+        <v>36.6</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>900</v>
@@ -1457,12 +1464,12 @@
       <c r="L9" s="3" t="n">
         <v>3103</v>
       </c>
-      <c r="M9" s="7" t="n">
-        <v>0.2232446043165468</v>
+      <c r="M9" s="8" t="n">
+        <v>22.3</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>우삼겹 2~3인</t>
         </is>
@@ -1485,8 +1492,8 @@
       <c r="G10" s="3" t="n">
         <v>11932</v>
       </c>
-      <c r="H10" s="7" t="n">
-        <v>0.4338909090909091</v>
+      <c r="H10" s="8" t="n">
+        <v>43.4</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>900</v>
@@ -1500,12 +1507,12 @@
       <c r="L10" s="3" t="n">
         <v>9084</v>
       </c>
-      <c r="M10" s="7" t="n">
-        <v>0.3427735849056604</v>
+      <c r="M10" s="8" t="n">
+        <v>34.3</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>우삼겹 3~4인</t>
         </is>
@@ -1528,8 +1535,8 @@
       <c r="G11" s="3" t="n">
         <v>15786</v>
       </c>
-      <c r="H11" s="7" t="n">
-        <v>0.4324931506849315</v>
+      <c r="H11" s="8" t="n">
+        <v>43.2</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>900</v>
@@ -1543,8 +1550,8 @@
       <c r="L11" s="3" t="n">
         <v>12576</v>
       </c>
-      <c r="M11" s="7" t="n">
-        <v>0.3542676056338028</v>
+      <c r="M11" s="8" t="n">
+        <v>35.4</v>
       </c>
     </row>
     <row r="12">
@@ -1553,11 +1560,11 @@
           <t>매출 가중 평균</t>
         </is>
       </c>
-      <c r="H12" s="7" t="n">
-        <v>0.4489675030851502</v>
-      </c>
-      <c r="M12" s="7" t="n">
-        <v>0.3514839124839125</v>
+      <c r="H12" s="8" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>35.1</v>
       </c>
     </row>
     <row r="13">
@@ -1762,20 +1769,20 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>영업시간 (h/일)</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="n">
+          <t>영업시간 (하루)</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>사장 근무 (h/월)</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="n">
+          <t>사장 근무 (월)</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
         <v>260</v>
       </c>
     </row>
@@ -1896,7 +1903,7 @@
           <t>영업이익 0원</t>
         </is>
       </c>
-      <c r="B36" t="n">
+      <c r="B36" s="10" t="n">
         <v>29</v>
       </c>
     </row>
@@ -1906,7 +1913,7 @@
           <t>사장 월 300만원 확보</t>
         </is>
       </c>
-      <c r="B37" t="n">
+      <c r="B37" s="10" t="n">
         <v>56</v>
       </c>
     </row>
@@ -1916,7 +1923,7 @@
           <t>사장 300만 + 투자금 24개월 회수</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="B38" s="10" t="n">
         <v>95</v>
       </c>
     </row>

</xml_diff>